<commit_message>
Week 4 Saturday: fix pass on the hiring interviewer's cold read
Q11's keyed option now says only what Amazon's letter says. Fourteen items
the interviewer read as medium are hardened with the read's own rewrites:
distractors that share the key's numbers and differ in judgment (Q4, Q6,
Q10, Q24, Q26, Q27, Q28, Q31), a claim title on the flattering denominator
in Q8, a wrong-unit check in Q12, a wrong-period check in Q13, and stems
that no longer name the method or the date (Q30, Q33). Q30's key accepts
part of the run-up in late October. Levels: 8 easy, 8 medium, 23 hard.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01M3TYrKwqBYtaKqFgbeoeQn
</commit_message>
<xml_diff>
--- a/content/W04/SAT/answer-key/C2_W04_SAT_item_analysis_TRAINER.xlsx
+++ b/content/W04/SAT/answer-key/C2_W04_SAT_item_analysis_TRAINER.xlsx
@@ -3252,7 +3252,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -3612,7 +3612,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Hard</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -3732,7 +3732,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -5112,7 +5112,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -5172,7 +5172,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -5232,7 +5232,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -5292,7 +5292,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -5352,7 +5352,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Easy</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">

</xml_diff>

<commit_message>
W04 SAT: the blind sitting's fixes, and five items back to Medium on its read
Exhibit 5E no longer prints "not a forecast" beside the plan line, which now sits in Q33's stem,
and every Q33 option says its six months held no Diwali. Q6 asks for two additions to the written
definition, and its wrong exclusion drops the remittance accounts the 2013 row names. Q14's option
c names the 64 lakh it moves to, Q39's two halves run the same length, Exhibit 5D leaves the spare
shipment's cost for the room to divide, and Exhibit 2A's role label prints whole. The keys give the
hidden weeks' dates and Q10's floor. Q6, Q12, Q31, Q33 and Q39 are Medium, as the sitting read
them; the paper holds 9 easy, 17 medium and 13 hard items, and the proofs assert that shape.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Xzgk1z5yvgqgEKKJve75mt
</commit_message>
<xml_diff>
--- a/content/W04/SAT/answer-key/C2_W04_SAT_item_analysis_TRAINER.xlsx
+++ b/content/W04/SAT/answer-key/C2_W04_SAT_item_analysis_TRAINER.xlsx
@@ -3432,7 +3432,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -3792,7 +3792,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -4932,7 +4932,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -5052,7 +5052,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -5412,7 +5412,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Hard</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">

</xml_diff>